<commit_message>
Cross-reference Overture Maps data for kebab/pizza/burger/sushi
Overture's place taxonomy has controlled categories matching these 4
target foods directly (doner_kebab, pizza_restaurant, burger_restaurant,
sushi_restaurant) - no LLM or web search needed for this signal. Matches
against existing venues by name+proximity to add confirmed target foods,
and adds genuinely new venues (88) that weren't in the OSM-derived set.

Tried before Google Places API since it's free and required no billing
setup; closed a meaningful chunk of the previously-unresolved gap.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/preprocessed/classifications.xlsx
+++ b/data/preprocessed/classifications.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N612"/>
+  <dimension ref="A1:N681"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2500,7 +2500,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>cafe_with_food; pub_with_food</t>
+          <t>cafe_with_food; pizzeria; pub_with_food</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2515,17 +2515,17 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>breakfast; soup; salad; dessert</t>
+          <t>breakfast; dessert; pizza; salad; soup</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Social media and restaurant listings indicate the venue serves local Moldovan-style food, including patisserie, breakfast, soup, salad, and dessert, with no evidence of specific international cuisines. The name and offerings suggest a local, home-style establishment.</t>
+          <t>Social media and restaurant listings indicate the venue serves local Moldovan-style food, including patisserie, breakfast, soup, salad, and dessert, with no evidence of specific international cuisines. The name and offerings suggest a local, home-style establishment. Overture Maps category match: pizza_restaurant (confidence 0.43, name match 0.89)</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>official_social (https://www.facebook.com/p/Moldovița-61560131927502/); reputable_listing (https://restaurantguru.com/Moldovita-Chisinau); official_social (https://www.facebook.com/moldovitapub/); official_social (https://www.instagram.com/simigeria.moldovita/)</t>
+          <t>official_social (https://www.facebook.com/p/Moldovița-61560131927502/); reputable_listing (https://restaurantguru.com/Moldovita-Chisinau); official_social (https://www.facebook.com/moldovitapub/); official_social (https://www.instagram.com/simigeria.moldovita/); other</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
@@ -11572,24 +11572,24 @@
       </c>
       <c r="F191" t="inlineStr">
         <is>
-          <t>fast_food; kebab_shop</t>
+          <t>burger_shop; fast_food; kebab_shop</t>
         </is>
       </c>
       <c r="G191" t="inlineStr"/>
       <c r="H191" t="inlineStr"/>
       <c r="I191" t="inlineStr">
         <is>
-          <t>kebab</t>
+          <t>burger; kebab</t>
         </is>
       </c>
       <c r="J191" t="inlineStr">
         <is>
-          <t>OSM cuisine tokens gave a clear food classification</t>
+          <t>OSM cuisine tokens gave a clear food classification Overture Maps category match: burger_restaurant, doner_kebab (confidence 0.99, name match 1.00)</t>
         </is>
       </c>
       <c r="K191" t="inlineStr">
         <is>
-          <t>osm</t>
+          <t>osm; other (https://kebabcity.md/)</t>
         </is>
       </c>
       <c r="L191" t="inlineStr"/>
@@ -12260,24 +12260,24 @@
       </c>
       <c r="F202" t="inlineStr">
         <is>
-          <t>pub_with_food; bar_with_food</t>
+          <t>bar_with_food; burger_shop; pub_with_food</t>
         </is>
       </c>
       <c r="G202" t="inlineStr"/>
       <c r="H202" t="inlineStr"/>
       <c r="I202" t="inlineStr">
         <is>
-          <t>salad; grill; beef_bowl</t>
+          <t>beef_bowl; burger; grill; salad</t>
         </is>
       </c>
       <c r="J202" t="inlineStr">
         <is>
-          <t>The menu includes beetroot carpaccio salad and lamb chop, indicating savory dishes. The venue is described as a craft beer bar with a fusion of flavors and full meal offerings. No specific cuisine or country is explicitly stated.</t>
+          <t>The menu includes beetroot carpaccio salad and lamb chop, indicating savory dishes. The venue is described as a craft beer bar with a fusion of flavors and full meal offerings. No specific cuisine or country is explicitly stated. Overture Maps category match: burger_restaurant (confidence 0.99, name match 1.00)</t>
         </is>
       </c>
       <c r="K202" t="inlineStr">
         <is>
-          <t>official_menu (https://restaurantguru.com/1516-by-RockScor-Brewery-Chisinau/menu); reputable_listing (https://g0.md/en/explore/1516-by-rockscor-brewery); delivery_platform (https://glovoapp.com/bs/md/chisinau/stores/1516-by-rockscor-brewery-ksn); osm</t>
+          <t>official_menu (https://restaurantguru.com/1516-by-RockScor-Brewery-Chisinau/menu); reputable_listing (https://g0.md/en/explore/1516-by-rockscor-brewery); delivery_platform (https://glovoapp.com/bs/md/chisinau/stores/1516-by-rockscor-brewery-ksn); osm; other (http://rockscor.md/)</t>
         </is>
       </c>
       <c r="L202" t="inlineStr">
@@ -13892,24 +13892,24 @@
       </c>
       <c r="F230" t="inlineStr">
         <is>
-          <t>pizzeria; restaurant</t>
+          <t>burger_shop; pizzeria; restaurant</t>
         </is>
       </c>
       <c r="G230" t="inlineStr"/>
       <c r="H230" t="inlineStr"/>
       <c r="I230" t="inlineStr">
         <is>
-          <t>pizza</t>
+          <t>burger; pizza</t>
         </is>
       </c>
       <c r="J230" t="inlineStr">
         <is>
-          <t>OSM cuisine tokens gave a clear food classification</t>
+          <t>OSM cuisine tokens gave a clear food classification Overture Maps category match: burger_restaurant, pizza_restaurant (confidence 0.99, name match 1.00)</t>
         </is>
       </c>
       <c r="K230" t="inlineStr">
         <is>
-          <t>osm</t>
+          <t>osm; other (https://doncezar.md)</t>
         </is>
       </c>
       <c r="L230" t="inlineStr"/>
@@ -18772,7 +18772,7 @@
       </c>
       <c r="F312" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>restaurant; sushi_restaurant</t>
         </is>
       </c>
       <c r="G312" t="inlineStr">
@@ -18781,15 +18781,19 @@
         </is>
       </c>
       <c r="H312" t="inlineStr"/>
-      <c r="I312" t="inlineStr"/>
+      <c r="I312" t="inlineStr">
+        <is>
+          <t>sushi</t>
+        </is>
+      </c>
       <c r="J312" t="inlineStr">
         <is>
-          <t>OSM cuisine tokens gave a clear food classification</t>
+          <t>OSM cuisine tokens gave a clear food classification Overture Maps category match: sushi_restaurant (confidence 1.00, name match 1.00)</t>
         </is>
       </c>
       <c r="K312" t="inlineStr">
         <is>
-          <t>osm</t>
+          <t>osm; other (http://www.momo.md/)</t>
         </is>
       </c>
       <c r="L312" t="inlineStr"/>
@@ -19328,7 +19332,7 @@
       </c>
       <c r="F321" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>restaurant; sushi_restaurant</t>
         </is>
       </c>
       <c r="G321" t="inlineStr">
@@ -19341,15 +19345,19 @@
           <t>Turkish</t>
         </is>
       </c>
-      <c r="I321" t="inlineStr"/>
+      <c r="I321" t="inlineStr">
+        <is>
+          <t>sushi</t>
+        </is>
+      </c>
       <c r="J321" t="inlineStr">
         <is>
-          <t>OSM cuisine tokens gave a clear food classification</t>
+          <t>OSM cuisine tokens gave a clear food classification Overture Maps category match: sushi_restaurant (confidence 0.99, name match 1.00)</t>
         </is>
       </c>
       <c r="K321" t="inlineStr">
         <is>
-          <t>osm</t>
+          <t>osm; other</t>
         </is>
       </c>
       <c r="L321" t="inlineStr"/>
@@ -20128,24 +20136,24 @@
       </c>
       <c r="F335" t="inlineStr">
         <is>
-          <t>fast_food; grill_house</t>
+          <t>burger_shop; fast_food; grill_house</t>
         </is>
       </c>
       <c r="G335" t="inlineStr"/>
       <c r="H335" t="inlineStr"/>
       <c r="I335" t="inlineStr">
         <is>
-          <t>grill</t>
+          <t>burger; grill</t>
         </is>
       </c>
       <c r="J335" t="inlineStr">
         <is>
-          <t>Beef House is a fast-food chain known for a rich selection of expertly prepared meat dishes, particularly grilled beef. It is described as a popular meat-focused restaurant in Chisinau, with no explicit mention of specific cuisines or regional origins.</t>
+          <t>Beef House is a fast-food chain known for a rich selection of expertly prepared meat dishes, particularly grilled beef. It is described as a popular meat-focused restaurant in Chisinau, with no explicit mention of specific cuisines or regional origins. Overture Maps category match: burger_restaurant (confidence 0.73, name match 1.00)</t>
         </is>
       </c>
       <c r="K335" t="inlineStr">
         <is>
-          <t>reputable_listing (https://www.tripadvisor.com/Restaurant_Review-g294456-d10400027-Reviews-Beef_House-Chisinau_Chisinau_District.html); reputable_listing (https://restaurantguru.com/Beef-House-Chisinau-2); osm</t>
+          <t>reputable_listing (https://www.tripadvisor.com/Restaurant_Review-g294456-d10400027-Reviews-Beef_House-Chisinau_Chisinau_District.html); reputable_listing (https://restaurantguru.com/Beef-House-Chisinau-2); osm; other</t>
         </is>
       </c>
       <c r="L335" t="inlineStr">
@@ -24896,24 +24904,24 @@
       </c>
       <c r="F417" t="inlineStr">
         <is>
-          <t>cafe_with_food</t>
+          <t>cafe_with_food; pizzeria</t>
         </is>
       </c>
       <c r="G417" t="inlineStr"/>
       <c r="H417" t="inlineStr"/>
       <c r="I417" t="inlineStr">
         <is>
-          <t>breakfast</t>
+          <t>breakfast; pizza</t>
         </is>
       </c>
       <c r="J417" t="inlineStr">
         <is>
-          <t>Menu and social media indicate breakfast offerings including smântână and caramel, with no explicit mention of specific cuisines or regional dishes beyond local breakfast items.</t>
+          <t>Menu and social media indicate breakfast offerings including smântână and caramel, with no explicit mention of specific cuisines or regional dishes beyond local breakfast items. Overture Maps category match: pizza_restaurant (confidence 0.29, name match 1.00)</t>
         </is>
       </c>
       <c r="K417" t="inlineStr">
         <is>
-          <t>official_menu (https://fr.restaurantguru.com/ANI-AMI-CAFE-Chisinau/menu); official_menu (https://de.restaurantguru.com/ANI-AMI-CAFE-Chisinau/menu); official_menu (https://es.restaurantguru.com/ANI-AMI-CAFE-Chisinau/menu); official_menu (https://ru.restaurantguru.com/ANI-AMI-CAFE-Chisinau/menu); official_social (https://www.facebook.com/ani.ami.cafe/)</t>
+          <t>official_menu (https://fr.restaurantguru.com/ANI-AMI-CAFE-Chisinau/menu); official_menu (https://de.restaurantguru.com/ANI-AMI-CAFE-Chisinau/menu); official_menu (https://es.restaurantguru.com/ANI-AMI-CAFE-Chisinau/menu); official_menu (https://ru.restaurantguru.com/ANI-AMI-CAFE-Chisinau/menu); official_social (https://www.facebook.com/ani.ami.cafe/); other (https://foodhouse.md/ru/ani-ami-cafe)</t>
         </is>
       </c>
       <c r="L417" t="inlineStr">
@@ -35800,7 +35808,7 @@
       </c>
       <c r="F598" t="inlineStr">
         <is>
-          <t>cafe_with_food</t>
+          <t>cafe_with_food; sushi_restaurant</t>
         </is>
       </c>
       <c r="G598" t="inlineStr">
@@ -35813,15 +35821,19 @@
           <t>Moldovan</t>
         </is>
       </c>
-      <c r="I598" t="inlineStr"/>
+      <c r="I598" t="inlineStr">
+        <is>
+          <t>sushi</t>
+        </is>
+      </c>
       <c r="J598" t="inlineStr">
         <is>
-          <t>Fortus Café is listed as a halal restaurant in Chisinau, Moldova, with a full menu and visitor reviews. The venue is categorized as a cafe with food service, and halal certification suggests local, regional cuisine. No specific dishes or cuisines are explicitly named in the menu descriptions.</t>
+          <t>Fortus Café is listed as a halal restaurant in Chisinau, Moldova, with a full menu and visitor reviews. The venue is categorized as a cafe with food service, and halal certification suggests local, regional cuisine. No specific dishes or cuisines are explicitly named in the menu descriptions. Overture Maps category match: sushi_restaurant (confidence 0.96, name match 1.00)</t>
         </is>
       </c>
       <c r="K598" t="inlineStr">
         <is>
-          <t>reputable_listing (https://fr.restaurantguru.com/Fortus-Chisinau); reputable_listing (https://halalfoodle.com/restaurants/moldova/chisinau/fortus-cafe-bulevardul-grigore-vieru-5); osm</t>
+          <t>reputable_listing (https://fr.restaurantguru.com/Fortus-Chisinau); reputable_listing (https://halalfoodle.com/restaurants/moldova/chisinau/fortus-cafe-bulevardul-grigore-vieru-5); osm; other (https://fortus.md/)</t>
         </is>
       </c>
       <c r="L598" t="inlineStr"/>
@@ -36700,6 +36712,3870 @@
         <v>28.890726</v>
       </c>
     </row>
+    <row r="613">
+      <c r="A613" t="inlineStr">
+        <is>
+          <t>overture/f344c7ac-550e-44b2-817d-07b318b33608</t>
+        </is>
+      </c>
+      <c r="B613" t="inlineStr">
+        <is>
+          <t>Max Kebab</t>
+        </is>
+      </c>
+      <c r="C613" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D613" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E613" t="inlineStr">
+        <is>
+          <t>limited_meal</t>
+        </is>
+      </c>
+      <c r="F613" t="inlineStr">
+        <is>
+          <t>kebab_shop</t>
+        </is>
+      </c>
+      <c r="G613" t="inlineStr"/>
+      <c r="H613" t="inlineStr"/>
+      <c r="I613" t="inlineStr">
+        <is>
+          <t>kebab</t>
+        </is>
+      </c>
+      <c r="J613" t="inlineStr">
+        <is>
+          <t>Overture Maps category: doner_kebab (confidence 0.65) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K613" t="inlineStr">
+        <is>
+          <t>other (https://maxkebab.md/?utm_source=ig&amp;utm_medium=social&amp;utm_content=link_in_bio&amp;fbclid=PAdGRleAPfPu9leHRuA2FlbQIxMQBzcnRjBmFwcF9pZA8xMjQwMjQ1NzQyODc0MTQAAacXA3-oYpMBHHs4pn7Ua2IoIXlNVxVq8vMsPbQmWJdjJWXbkZlGrSqILCYf2Q_aem_behP0YioHZgvn0DyxoL06w)</t>
+        </is>
+      </c>
+      <c r="L613" t="inlineStr"/>
+      <c r="M613" t="n">
+        <v>46.95165439</v>
+      </c>
+      <c r="N613" t="n">
+        <v>28.77141619</v>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" t="inlineStr">
+        <is>
+          <t>overture/c8188b2d-92f0-4746-b1b9-03bf240d79f1</t>
+        </is>
+      </c>
+      <c r="B614" t="inlineStr">
+        <is>
+          <t>Casa della Pizza</t>
+        </is>
+      </c>
+      <c r="C614" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D614" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E614" t="inlineStr">
+        <is>
+          <t>full_meal</t>
+        </is>
+      </c>
+      <c r="F614" t="inlineStr">
+        <is>
+          <t>pizzeria</t>
+        </is>
+      </c>
+      <c r="G614" t="inlineStr"/>
+      <c r="H614" t="inlineStr"/>
+      <c r="I614" t="inlineStr">
+        <is>
+          <t>pizza</t>
+        </is>
+      </c>
+      <c r="J614" t="inlineStr">
+        <is>
+          <t>Overture Maps category: pizza_restaurant (confidence 0.99) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K614" t="inlineStr">
+        <is>
+          <t>other (http://www.casadellapizza.md/)</t>
+        </is>
+      </c>
+      <c r="L614" t="inlineStr"/>
+      <c r="M614" t="n">
+        <v>46.95233697</v>
+      </c>
+      <c r="N614" t="n">
+        <v>28.77155373</v>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" t="inlineStr">
+        <is>
+          <t>overture/95a070ef-9766-4f50-981f-1e3e74317d20</t>
+        </is>
+      </c>
+      <c r="B615" t="inlineStr">
+        <is>
+          <t>Pizza Mania</t>
+        </is>
+      </c>
+      <c r="C615" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D615" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E615" t="inlineStr">
+        <is>
+          <t>full_meal</t>
+        </is>
+      </c>
+      <c r="F615" t="inlineStr">
+        <is>
+          <t>pizzeria</t>
+        </is>
+      </c>
+      <c r="G615" t="inlineStr"/>
+      <c r="H615" t="inlineStr"/>
+      <c r="I615" t="inlineStr">
+        <is>
+          <t>pizza</t>
+        </is>
+      </c>
+      <c r="J615" t="inlineStr">
+        <is>
+          <t>Overture Maps category: pizza_restaurant (confidence 0.54) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K615" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="L615" t="inlineStr"/>
+      <c r="M615" t="n">
+        <v>46.97645179</v>
+      </c>
+      <c r="N615" t="n">
+        <v>28.76825429</v>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" t="inlineStr">
+        <is>
+          <t>overture/1a9811f9-649a-47f2-ae15-4295416db933</t>
+        </is>
+      </c>
+      <c r="B616" t="inlineStr">
+        <is>
+          <t>Гори Шишка</t>
+        </is>
+      </c>
+      <c r="C616" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D616" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E616" t="inlineStr">
+        <is>
+          <t>full_meal</t>
+        </is>
+      </c>
+      <c r="F616" t="inlineStr">
+        <is>
+          <t>sushi_restaurant</t>
+        </is>
+      </c>
+      <c r="G616" t="inlineStr"/>
+      <c r="H616" t="inlineStr"/>
+      <c r="I616" t="inlineStr">
+        <is>
+          <t>sushi</t>
+        </is>
+      </c>
+      <c r="J616" t="inlineStr">
+        <is>
+          <t>Overture Maps category: sushi_restaurant (confidence 0.94) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K616" t="inlineStr">
+        <is>
+          <t>other (http://gori-shishka.club/)</t>
+        </is>
+      </c>
+      <c r="L616" t="inlineStr"/>
+      <c r="M616" t="n">
+        <v>46.976914443857</v>
+      </c>
+      <c r="N616" t="n">
+        <v>28.857886791229</v>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" t="inlineStr">
+        <is>
+          <t>overture/31b11cde-fa90-4878-aca4-c36192cb17e8</t>
+        </is>
+      </c>
+      <c r="B617" t="inlineStr">
+        <is>
+          <t>Beer Park</t>
+        </is>
+      </c>
+      <c r="C617" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D617" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E617" t="inlineStr">
+        <is>
+          <t>full_meal</t>
+        </is>
+      </c>
+      <c r="F617" t="inlineStr">
+        <is>
+          <t>pizzeria</t>
+        </is>
+      </c>
+      <c r="G617" t="inlineStr"/>
+      <c r="H617" t="inlineStr"/>
+      <c r="I617" t="inlineStr">
+        <is>
+          <t>pizza</t>
+        </is>
+      </c>
+      <c r="J617" t="inlineStr">
+        <is>
+          <t>Overture Maps category: pizza_restaurant (confidence 0.90) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K617" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="L617" t="inlineStr"/>
+      <c r="M617" t="n">
+        <v>46.9766016</v>
+      </c>
+      <c r="N617" t="n">
+        <v>28.8550736</v>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" t="inlineStr">
+        <is>
+          <t>overture/c37a2d5e-2a76-4643-9f0a-fca2717e226f</t>
+        </is>
+      </c>
+      <c r="B618" t="inlineStr">
+        <is>
+          <t>СУШИ Мания</t>
+        </is>
+      </c>
+      <c r="C618" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D618" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E618" t="inlineStr">
+        <is>
+          <t>full_meal</t>
+        </is>
+      </c>
+      <c r="F618" t="inlineStr">
+        <is>
+          <t>sushi_restaurant</t>
+        </is>
+      </c>
+      <c r="G618" t="inlineStr"/>
+      <c r="H618" t="inlineStr"/>
+      <c r="I618" t="inlineStr">
+        <is>
+          <t>sushi</t>
+        </is>
+      </c>
+      <c r="J618" t="inlineStr">
+        <is>
+          <t>Overture Maps category: sushi_restaurant (confidence 0.58) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K618" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="L618" t="inlineStr"/>
+      <c r="M618" t="n">
+        <v>46.97895</v>
+      </c>
+      <c r="N618" t="n">
+        <v>28.85512</v>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" t="inlineStr">
+        <is>
+          <t>overture/7e68c3a3-664e-43a9-a259-7fbdc7cf29e1</t>
+        </is>
+      </c>
+      <c r="B619" t="inlineStr">
+        <is>
+          <t>MR.PUB'S_kebab&amp;burger</t>
+        </is>
+      </c>
+      <c r="C619" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D619" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E619" t="inlineStr">
+        <is>
+          <t>limited_meal</t>
+        </is>
+      </c>
+      <c r="F619" t="inlineStr">
+        <is>
+          <t>burger_shop</t>
+        </is>
+      </c>
+      <c r="G619" t="inlineStr"/>
+      <c r="H619" t="inlineStr"/>
+      <c r="I619" t="inlineStr">
+        <is>
+          <t>burger</t>
+        </is>
+      </c>
+      <c r="J619" t="inlineStr">
+        <is>
+          <t>Overture Maps category: burger_restaurant (confidence 0.59) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K619" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="L619" t="inlineStr"/>
+      <c r="M619" t="n">
+        <v>46.97865296536</v>
+      </c>
+      <c r="N619" t="n">
+        <v>28.855577409267</v>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" t="inlineStr">
+        <is>
+          <t>overture/6b9b931b-ac40-44f2-8ddd-b0928f3fa481</t>
+        </is>
+      </c>
+      <c r="B620" t="inlineStr">
+        <is>
+          <t>Pizza4you</t>
+        </is>
+      </c>
+      <c r="C620" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D620" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E620" t="inlineStr">
+        <is>
+          <t>full_meal</t>
+        </is>
+      </c>
+      <c r="F620" t="inlineStr">
+        <is>
+          <t>pizzeria</t>
+        </is>
+      </c>
+      <c r="G620" t="inlineStr"/>
+      <c r="H620" t="inlineStr"/>
+      <c r="I620" t="inlineStr">
+        <is>
+          <t>pizza</t>
+        </is>
+      </c>
+      <c r="J620" t="inlineStr">
+        <is>
+          <t>Overture Maps category: pizza_restaurant (confidence 0.79) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K620" t="inlineStr">
+        <is>
+          <t>other (http://pizza4you.md/)</t>
+        </is>
+      </c>
+      <c r="L620" t="inlineStr"/>
+      <c r="M620" t="n">
+        <v>46.98148205951</v>
+      </c>
+      <c r="N620" t="n">
+        <v>28.850022554398</v>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" t="inlineStr">
+        <is>
+          <t>overture/b81b3b76-9e76-4167-8857-f7b134fecc86</t>
+        </is>
+      </c>
+      <c r="B621" t="inlineStr">
+        <is>
+          <t>Rotana restaurant Cofe</t>
+        </is>
+      </c>
+      <c r="C621" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D621" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E621" t="inlineStr">
+        <is>
+          <t>limited_meal</t>
+        </is>
+      </c>
+      <c r="F621" t="inlineStr">
+        <is>
+          <t>kebab_shop</t>
+        </is>
+      </c>
+      <c r="G621" t="inlineStr"/>
+      <c r="H621" t="inlineStr"/>
+      <c r="I621" t="inlineStr">
+        <is>
+          <t>kebab</t>
+        </is>
+      </c>
+      <c r="J621" t="inlineStr">
+        <is>
+          <t>Overture Maps category: doner_kebab (confidence 0.56) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K621" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="L621" t="inlineStr"/>
+      <c r="M621" t="n">
+        <v>46.981978</v>
+      </c>
+      <c r="N621" t="n">
+        <v>28.849714</v>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" t="inlineStr">
+        <is>
+          <t>overture/30501a5a-95a7-45e1-918b-e058c4d677c3</t>
+        </is>
+      </c>
+      <c r="B622" t="inlineStr">
+        <is>
+          <t>Andy's Restaurant</t>
+        </is>
+      </c>
+      <c r="C622" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D622" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E622" t="inlineStr">
+        <is>
+          <t>full_meal</t>
+        </is>
+      </c>
+      <c r="F622" t="inlineStr">
+        <is>
+          <t>pizzeria</t>
+        </is>
+      </c>
+      <c r="G622" t="inlineStr"/>
+      <c r="H622" t="inlineStr"/>
+      <c r="I622" t="inlineStr">
+        <is>
+          <t>pizza</t>
+        </is>
+      </c>
+      <c r="J622" t="inlineStr">
+        <is>
+          <t>Overture Maps category: pizza_restaurant (confidence 0.99) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K622" t="inlineStr">
+        <is>
+          <t>other (https://www.andys.md)</t>
+        </is>
+      </c>
+      <c r="L622" t="inlineStr"/>
+      <c r="M622" t="n">
+        <v>46.98468956</v>
+      </c>
+      <c r="N622" t="n">
+        <v>28.85879607</v>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" t="inlineStr">
+        <is>
+          <t>overture/0f4ed3c8-65f6-43e2-a8bc-302093a3dc5d</t>
+        </is>
+      </c>
+      <c r="B623" t="inlineStr">
+        <is>
+          <t>Starkebab</t>
+        </is>
+      </c>
+      <c r="C623" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D623" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E623" t="inlineStr">
+        <is>
+          <t>limited_meal</t>
+        </is>
+      </c>
+      <c r="F623" t="inlineStr">
+        <is>
+          <t>kebab_shop</t>
+        </is>
+      </c>
+      <c r="G623" t="inlineStr"/>
+      <c r="H623" t="inlineStr"/>
+      <c r="I623" t="inlineStr">
+        <is>
+          <t>kebab</t>
+        </is>
+      </c>
+      <c r="J623" t="inlineStr">
+        <is>
+          <t>Overture Maps category: doner_kebab (confidence 0.70) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K623" t="inlineStr">
+        <is>
+          <t>other (http://www.starkebab.md/)</t>
+        </is>
+      </c>
+      <c r="L623" t="inlineStr"/>
+      <c r="M623" t="n">
+        <v>47.00421068</v>
+      </c>
+      <c r="N623" t="n">
+        <v>28.84094367</v>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" t="inlineStr">
+        <is>
+          <t>overture/6ef2e82f-8e76-4302-aa2d-bf6dd4a561ab</t>
+        </is>
+      </c>
+      <c r="B624" t="inlineStr">
+        <is>
+          <t>Yum Yum Sushi</t>
+        </is>
+      </c>
+      <c r="C624" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D624" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E624" t="inlineStr">
+        <is>
+          <t>full_meal</t>
+        </is>
+      </c>
+      <c r="F624" t="inlineStr">
+        <is>
+          <t>sushi_restaurant</t>
+        </is>
+      </c>
+      <c r="G624" t="inlineStr"/>
+      <c r="H624" t="inlineStr"/>
+      <c r="I624" t="inlineStr">
+        <is>
+          <t>sushi</t>
+        </is>
+      </c>
+      <c r="J624" t="inlineStr">
+        <is>
+          <t>Overture Maps category: sushi_restaurant (confidence 0.93) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K624" t="inlineStr">
+        <is>
+          <t>other (https://yum-yum.md/)</t>
+        </is>
+      </c>
+      <c r="L624" t="inlineStr"/>
+      <c r="M624" t="n">
+        <v>47.00070442</v>
+      </c>
+      <c r="N624" t="n">
+        <v>28.85981239</v>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" t="inlineStr">
+        <is>
+          <t>overture/91b32d93-7fee-4cd7-ab85-b4d511a500ce</t>
+        </is>
+      </c>
+      <c r="B625" t="inlineStr">
+        <is>
+          <t>Pegas Burger Cafe</t>
+        </is>
+      </c>
+      <c r="C625" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D625" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E625" t="inlineStr">
+        <is>
+          <t>limited_meal</t>
+        </is>
+      </c>
+      <c r="F625" t="inlineStr">
+        <is>
+          <t>burger_shop</t>
+        </is>
+      </c>
+      <c r="G625" t="inlineStr"/>
+      <c r="H625" t="inlineStr"/>
+      <c r="I625" t="inlineStr">
+        <is>
+          <t>burger</t>
+        </is>
+      </c>
+      <c r="J625" t="inlineStr">
+        <is>
+          <t>Overture Maps category: burger_restaurant (confidence 0.99) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K625" t="inlineStr">
+        <is>
+          <t>other (http://www.pb.md/)</t>
+        </is>
+      </c>
+      <c r="L625" t="inlineStr"/>
+      <c r="M625" t="n">
+        <v>46.99812235</v>
+      </c>
+      <c r="N625" t="n">
+        <v>28.85817168</v>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" t="inlineStr">
+        <is>
+          <t>overture/2af17f8d-c1cd-466a-b47f-1a1e35696d61</t>
+        </is>
+      </c>
+      <c r="B626" t="inlineStr">
+        <is>
+          <t>Zelinski.md</t>
+        </is>
+      </c>
+      <c r="C626" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D626" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E626" t="inlineStr">
+        <is>
+          <t>full_meal</t>
+        </is>
+      </c>
+      <c r="F626" t="inlineStr">
+        <is>
+          <t>sushi_restaurant</t>
+        </is>
+      </c>
+      <c r="G626" t="inlineStr"/>
+      <c r="H626" t="inlineStr"/>
+      <c r="I626" t="inlineStr">
+        <is>
+          <t>sushi</t>
+        </is>
+      </c>
+      <c r="J626" t="inlineStr">
+        <is>
+          <t>Overture Maps category: sushi_restaurant (confidence 0.68) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K626" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="L626" t="inlineStr"/>
+      <c r="M626" t="n">
+        <v>46.99484</v>
+      </c>
+      <c r="N626" t="n">
+        <v>28.85413</v>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" t="inlineStr">
+        <is>
+          <t>overture/37df7f05-d14f-4aba-989b-6af020d0672b</t>
+        </is>
+      </c>
+      <c r="B627" t="inlineStr">
+        <is>
+          <t>Kebab House</t>
+        </is>
+      </c>
+      <c r="C627" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D627" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E627" t="inlineStr">
+        <is>
+          <t>limited_meal</t>
+        </is>
+      </c>
+      <c r="F627" t="inlineStr">
+        <is>
+          <t>kebab_shop</t>
+        </is>
+      </c>
+      <c r="G627" t="inlineStr"/>
+      <c r="H627" t="inlineStr"/>
+      <c r="I627" t="inlineStr">
+        <is>
+          <t>kebab</t>
+        </is>
+      </c>
+      <c r="J627" t="inlineStr">
+        <is>
+          <t>Overture Maps category: doner_kebab (confidence 0.89) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K627" t="inlineStr">
+        <is>
+          <t>other (http://kebabhouse.com/)</t>
+        </is>
+      </c>
+      <c r="L627" t="inlineStr"/>
+      <c r="M627" t="n">
+        <v>46.99142</v>
+      </c>
+      <c r="N627" t="n">
+        <v>28.84483</v>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" t="inlineStr">
+        <is>
+          <t>overture/68e6db58-2e46-49a2-afe7-6491da5acd96</t>
+        </is>
+      </c>
+      <c r="B628" t="inlineStr">
+        <is>
+          <t>Ciao Steak</t>
+        </is>
+      </c>
+      <c r="C628" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D628" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E628" t="inlineStr">
+        <is>
+          <t>full_meal</t>
+        </is>
+      </c>
+      <c r="F628" t="inlineStr">
+        <is>
+          <t>pizzeria</t>
+        </is>
+      </c>
+      <c r="G628" t="inlineStr"/>
+      <c r="H628" t="inlineStr"/>
+      <c r="I628" t="inlineStr">
+        <is>
+          <t>pizza</t>
+        </is>
+      </c>
+      <c r="J628" t="inlineStr">
+        <is>
+          <t>Overture Maps category: pizza_restaurant (confidence 0.58) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K628" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="L628" t="inlineStr"/>
+      <c r="M628" t="n">
+        <v>46.99535</v>
+      </c>
+      <c r="N628" t="n">
+        <v>28.82832</v>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" t="inlineStr">
+        <is>
+          <t>overture/b99d93c6-6667-4501-bde8-9178a6064efc</t>
+        </is>
+      </c>
+      <c r="B629" t="inlineStr">
+        <is>
+          <t>Суши-бар «Токио»</t>
+        </is>
+      </c>
+      <c r="C629" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D629" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E629" t="inlineStr">
+        <is>
+          <t>full_meal</t>
+        </is>
+      </c>
+      <c r="F629" t="inlineStr">
+        <is>
+          <t>sushi_restaurant</t>
+        </is>
+      </c>
+      <c r="G629" t="inlineStr"/>
+      <c r="H629" t="inlineStr"/>
+      <c r="I629" t="inlineStr">
+        <is>
+          <t>sushi</t>
+        </is>
+      </c>
+      <c r="J629" t="inlineStr">
+        <is>
+          <t>Overture Maps category: sushi_restaurant (confidence 0.62) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K629" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="L629" t="inlineStr"/>
+      <c r="M629" t="n">
+        <v>46.98923</v>
+      </c>
+      <c r="N629" t="n">
+        <v>28.82717</v>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" t="inlineStr">
+        <is>
+          <t>overture/be0aae04-cfa4-466a-9d6b-161b9c31b736</t>
+        </is>
+      </c>
+      <c r="B630" t="inlineStr">
+        <is>
+          <t>Black Angus Burger</t>
+        </is>
+      </c>
+      <c r="C630" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D630" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E630" t="inlineStr">
+        <is>
+          <t>limited_meal</t>
+        </is>
+      </c>
+      <c r="F630" t="inlineStr">
+        <is>
+          <t>burger_shop</t>
+        </is>
+      </c>
+      <c r="G630" t="inlineStr"/>
+      <c r="H630" t="inlineStr"/>
+      <c r="I630" t="inlineStr">
+        <is>
+          <t>burger</t>
+        </is>
+      </c>
+      <c r="J630" t="inlineStr">
+        <is>
+          <t>Overture Maps category: burger_restaurant (confidence 0.56) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K630" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="L630" t="inlineStr"/>
+      <c r="M630" t="n">
+        <v>46.98898313</v>
+      </c>
+      <c r="N630" t="n">
+        <v>28.85246585</v>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" t="inlineStr">
+        <is>
+          <t>overture/954399de-89b6-4466-8856-677d354612ef</t>
+        </is>
+      </c>
+      <c r="B631" t="inlineStr">
+        <is>
+          <t>MML Food</t>
+        </is>
+      </c>
+      <c r="C631" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D631" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E631" t="inlineStr">
+        <is>
+          <t>limited_meal</t>
+        </is>
+      </c>
+      <c r="F631" t="inlineStr">
+        <is>
+          <t>kebab_shop</t>
+        </is>
+      </c>
+      <c r="G631" t="inlineStr"/>
+      <c r="H631" t="inlineStr"/>
+      <c r="I631" t="inlineStr">
+        <is>
+          <t>kebab</t>
+        </is>
+      </c>
+      <c r="J631" t="inlineStr">
+        <is>
+          <t>Overture Maps category: doner_kebab (confidence 0.71) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K631" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="L631" t="inlineStr"/>
+      <c r="M631" t="n">
+        <v>46.98946623</v>
+      </c>
+      <c r="N631" t="n">
+        <v>28.85806419</v>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" t="inlineStr">
+        <is>
+          <t>overture/2eae6163-e36c-41d0-97cd-a81feec6e573</t>
+        </is>
+      </c>
+      <c r="B632" t="inlineStr">
+        <is>
+          <t>Panifico Pizza</t>
+        </is>
+      </c>
+      <c r="C632" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D632" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E632" t="inlineStr">
+        <is>
+          <t>full_meal</t>
+        </is>
+      </c>
+      <c r="F632" t="inlineStr">
+        <is>
+          <t>pizzeria</t>
+        </is>
+      </c>
+      <c r="G632" t="inlineStr"/>
+      <c r="H632" t="inlineStr"/>
+      <c r="I632" t="inlineStr">
+        <is>
+          <t>pizza</t>
+        </is>
+      </c>
+      <c r="J632" t="inlineStr">
+        <is>
+          <t>Overture Maps category: pizza_restaurant (confidence 0.97) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K632" t="inlineStr">
+        <is>
+          <t>other (http://panifico.md/)</t>
+        </is>
+      </c>
+      <c r="L632" t="inlineStr"/>
+      <c r="M632" t="n">
+        <v>46.9893685</v>
+      </c>
+      <c r="N632" t="n">
+        <v>28.85858245</v>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" t="inlineStr">
+        <is>
+          <t>overture/f48dcdc0-0b7f-4e5e-9bad-781f727ab2db</t>
+        </is>
+      </c>
+      <c r="B633" t="inlineStr">
+        <is>
+          <t>San Sushi</t>
+        </is>
+      </c>
+      <c r="C633" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D633" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E633" t="inlineStr">
+        <is>
+          <t>full_meal</t>
+        </is>
+      </c>
+      <c r="F633" t="inlineStr">
+        <is>
+          <t>sushi_restaurant</t>
+        </is>
+      </c>
+      <c r="G633" t="inlineStr"/>
+      <c r="H633" t="inlineStr"/>
+      <c r="I633" t="inlineStr">
+        <is>
+          <t>sushi</t>
+        </is>
+      </c>
+      <c r="J633" t="inlineStr">
+        <is>
+          <t>Overture Maps category: sushi_restaurant (confidence 1.00) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K633" t="inlineStr">
+        <is>
+          <t>other (http://sansushi.md/)</t>
+        </is>
+      </c>
+      <c r="L633" t="inlineStr"/>
+      <c r="M633" t="n">
+        <v>46.98664732</v>
+      </c>
+      <c r="N633" t="n">
+        <v>28.86811142</v>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" t="inlineStr">
+        <is>
+          <t>overture/66888f26-ebe5-4121-82c2-e643f99a2ff5</t>
+        </is>
+      </c>
+      <c r="B634" t="inlineStr">
+        <is>
+          <t>XEDA</t>
+        </is>
+      </c>
+      <c r="C634" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D634" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E634" t="inlineStr">
+        <is>
+          <t>limited_meal</t>
+        </is>
+      </c>
+      <c r="F634" t="inlineStr">
+        <is>
+          <t>burger_shop</t>
+        </is>
+      </c>
+      <c r="G634" t="inlineStr"/>
+      <c r="H634" t="inlineStr"/>
+      <c r="I634" t="inlineStr">
+        <is>
+          <t>burger</t>
+        </is>
+      </c>
+      <c r="J634" t="inlineStr">
+        <is>
+          <t>Overture Maps category: burger_restaurant (confidence 0.64) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K634" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="L634" t="inlineStr"/>
+      <c r="M634" t="n">
+        <v>46.98036</v>
+      </c>
+      <c r="N634" t="n">
+        <v>28.87465</v>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" t="inlineStr">
+        <is>
+          <t>overture/1eb42a8a-e28e-4cb2-9a15-90dbce29feac</t>
+        </is>
+      </c>
+      <c r="B635" t="inlineStr">
+        <is>
+          <t>Black Goose</t>
+        </is>
+      </c>
+      <c r="C635" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D635" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E635" t="inlineStr">
+        <is>
+          <t>full_meal</t>
+        </is>
+      </c>
+      <c r="F635" t="inlineStr">
+        <is>
+          <t>pizzeria</t>
+        </is>
+      </c>
+      <c r="G635" t="inlineStr"/>
+      <c r="H635" t="inlineStr"/>
+      <c r="I635" t="inlineStr">
+        <is>
+          <t>pizza</t>
+        </is>
+      </c>
+      <c r="J635" t="inlineStr">
+        <is>
+          <t>Overture Maps category: pizza_restaurant (confidence 0.77) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K635" t="inlineStr">
+        <is>
+          <t>other (https://blackgoose.md)</t>
+        </is>
+      </c>
+      <c r="L635" t="inlineStr"/>
+      <c r="M635" t="n">
+        <v>46.97731522382762</v>
+      </c>
+      <c r="N635" t="n">
+        <v>28.87077480554581</v>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" t="inlineStr">
+        <is>
+          <t>overture/cfd32712-3c42-434b-b01e-23cab3786186</t>
+        </is>
+      </c>
+      <c r="B636" t="inlineStr">
+        <is>
+          <t>Torro Burgers</t>
+        </is>
+      </c>
+      <c r="C636" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D636" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E636" t="inlineStr">
+        <is>
+          <t>limited_meal</t>
+        </is>
+      </c>
+      <c r="F636" t="inlineStr">
+        <is>
+          <t>burger_shop</t>
+        </is>
+      </c>
+      <c r="G636" t="inlineStr"/>
+      <c r="H636" t="inlineStr"/>
+      <c r="I636" t="inlineStr">
+        <is>
+          <t>burger</t>
+        </is>
+      </c>
+      <c r="J636" t="inlineStr">
+        <is>
+          <t>Overture Maps category: burger_restaurant (confidence 0.84) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K636" t="inlineStr">
+        <is>
+          <t>other (http://www.torroburgers.md/)</t>
+        </is>
+      </c>
+      <c r="L636" t="inlineStr"/>
+      <c r="M636" t="n">
+        <v>47.04219</v>
+      </c>
+      <c r="N636" t="n">
+        <v>28.76098</v>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" t="inlineStr">
+        <is>
+          <t>overture/ddb4d75c-f615-477c-9153-42488e158e0f</t>
+        </is>
+      </c>
+      <c r="B637" t="inlineStr">
+        <is>
+          <t>Ritus</t>
+        </is>
+      </c>
+      <c r="C637" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D637" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E637" t="inlineStr">
+        <is>
+          <t>full_meal</t>
+        </is>
+      </c>
+      <c r="F637" t="inlineStr">
+        <is>
+          <t>sushi_restaurant</t>
+        </is>
+      </c>
+      <c r="G637" t="inlineStr"/>
+      <c r="H637" t="inlineStr"/>
+      <c r="I637" t="inlineStr">
+        <is>
+          <t>sushi</t>
+        </is>
+      </c>
+      <c r="J637" t="inlineStr">
+        <is>
+          <t>Overture Maps category: sushi_restaurant (confidence 0.98) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K637" t="inlineStr">
+        <is>
+          <t>other (https://ritus.md/)</t>
+        </is>
+      </c>
+      <c r="L637" t="inlineStr"/>
+      <c r="M637" t="n">
+        <v>47.06244867</v>
+      </c>
+      <c r="N637" t="n">
+        <v>28.83509174</v>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" t="inlineStr">
+        <is>
+          <t>overture/9cf0593c-0c3e-4709-839a-54c7c47b8583</t>
+        </is>
+      </c>
+      <c r="B638" t="inlineStr">
+        <is>
+          <t>Star Kebab</t>
+        </is>
+      </c>
+      <c r="C638" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D638" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E638" t="inlineStr">
+        <is>
+          <t>limited_meal</t>
+        </is>
+      </c>
+      <c r="F638" t="inlineStr">
+        <is>
+          <t>kebab_shop</t>
+        </is>
+      </c>
+      <c r="G638" t="inlineStr"/>
+      <c r="H638" t="inlineStr"/>
+      <c r="I638" t="inlineStr">
+        <is>
+          <t>kebab</t>
+        </is>
+      </c>
+      <c r="J638" t="inlineStr">
+        <is>
+          <t>Overture Maps category: doner_kebab (confidence 0.77) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K638" t="inlineStr">
+        <is>
+          <t>other (https://starkebab.md)</t>
+        </is>
+      </c>
+      <c r="L638" t="inlineStr"/>
+      <c r="M638" t="n">
+        <v>47.071361105584</v>
+      </c>
+      <c r="N638" t="n">
+        <v>28.88871610164642</v>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" t="inlineStr">
+        <is>
+          <t>overture/b00b4e3c-4680-4138-8721-973975a6d8be</t>
+        </is>
+      </c>
+      <c r="B639" t="inlineStr">
+        <is>
+          <t>Do Cafe</t>
+        </is>
+      </c>
+      <c r="C639" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D639" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E639" t="inlineStr">
+        <is>
+          <t>full_meal</t>
+        </is>
+      </c>
+      <c r="F639" t="inlineStr">
+        <is>
+          <t>pizzeria</t>
+        </is>
+      </c>
+      <c r="G639" t="inlineStr"/>
+      <c r="H639" t="inlineStr"/>
+      <c r="I639" t="inlineStr">
+        <is>
+          <t>pizza</t>
+        </is>
+      </c>
+      <c r="J639" t="inlineStr">
+        <is>
+          <t>Overture Maps category: pizza_restaurant (confidence 0.94) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K639" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="L639" t="inlineStr"/>
+      <c r="M639" t="n">
+        <v>47.0499866</v>
+      </c>
+      <c r="N639" t="n">
+        <v>28.88966396</v>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" t="inlineStr">
+        <is>
+          <t>overture/4f8d3468-543f-4ccf-a883-7dd181139967</t>
+        </is>
+      </c>
+      <c r="B640" t="inlineStr">
+        <is>
+          <t>SUSHKA</t>
+        </is>
+      </c>
+      <c r="C640" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D640" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E640" t="inlineStr">
+        <is>
+          <t>full_meal</t>
+        </is>
+      </c>
+      <c r="F640" t="inlineStr">
+        <is>
+          <t>sushi_restaurant</t>
+        </is>
+      </c>
+      <c r="G640" t="inlineStr"/>
+      <c r="H640" t="inlineStr"/>
+      <c r="I640" t="inlineStr">
+        <is>
+          <t>sushi</t>
+        </is>
+      </c>
+      <c r="J640" t="inlineStr">
+        <is>
+          <t>Overture Maps category: sushi_restaurant (confidence 0.78) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K640" t="inlineStr">
+        <is>
+          <t>other (http://sushka.md/)</t>
+        </is>
+      </c>
+      <c r="L640" t="inlineStr"/>
+      <c r="M640" t="n">
+        <v>47.05134919774205</v>
+      </c>
+      <c r="N640" t="n">
+        <v>28.86360565092732</v>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" t="inlineStr">
+        <is>
+          <t>overture/1f97d580-e262-4d69-92f8-ef653406a1e2</t>
+        </is>
+      </c>
+      <c r="B641" t="inlineStr">
+        <is>
+          <t>Pizza9</t>
+        </is>
+      </c>
+      <c r="C641" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D641" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E641" t="inlineStr">
+        <is>
+          <t>full_meal</t>
+        </is>
+      </c>
+      <c r="F641" t="inlineStr">
+        <is>
+          <t>pizzeria</t>
+        </is>
+      </c>
+      <c r="G641" t="inlineStr"/>
+      <c r="H641" t="inlineStr"/>
+      <c r="I641" t="inlineStr">
+        <is>
+          <t>pizza</t>
+        </is>
+      </c>
+      <c r="J641" t="inlineStr">
+        <is>
+          <t>Overture Maps category: pizza_restaurant (confidence 0.66) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K641" t="inlineStr">
+        <is>
+          <t>other (http://www.pizza9.md/)</t>
+        </is>
+      </c>
+      <c r="L641" t="inlineStr"/>
+      <c r="M641" t="n">
+        <v>47.04394187</v>
+      </c>
+      <c r="N641" t="n">
+        <v>28.8436766</v>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" t="inlineStr">
+        <is>
+          <t>overture/5ee008c8-9c80-4a17-aec5-1ab749779aeb</t>
+        </is>
+      </c>
+      <c r="B642" t="inlineStr">
+        <is>
+          <t>Corso Pizza</t>
+        </is>
+      </c>
+      <c r="C642" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D642" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E642" t="inlineStr">
+        <is>
+          <t>full_meal</t>
+        </is>
+      </c>
+      <c r="F642" t="inlineStr">
+        <is>
+          <t>pizzeria</t>
+        </is>
+      </c>
+      <c r="G642" t="inlineStr"/>
+      <c r="H642" t="inlineStr"/>
+      <c r="I642" t="inlineStr">
+        <is>
+          <t>pizza</t>
+        </is>
+      </c>
+      <c r="J642" t="inlineStr">
+        <is>
+          <t>Overture Maps category: pizza_restaurant (confidence 0.99) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K642" t="inlineStr">
+        <is>
+          <t>other (http://www.cuptorulculemne.md)</t>
+        </is>
+      </c>
+      <c r="L642" t="inlineStr"/>
+      <c r="M642" t="n">
+        <v>47.04477474</v>
+      </c>
+      <c r="N642" t="n">
+        <v>28.88233537</v>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" t="inlineStr">
+        <is>
+          <t>overture/e78d2b6f-3702-4b0b-999c-1b64a2399226</t>
+        </is>
+      </c>
+      <c r="B643" t="inlineStr">
+        <is>
+          <t>Kamora Burger</t>
+        </is>
+      </c>
+      <c r="C643" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D643" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E643" t="inlineStr">
+        <is>
+          <t>limited_meal</t>
+        </is>
+      </c>
+      <c r="F643" t="inlineStr">
+        <is>
+          <t>burger_shop</t>
+        </is>
+      </c>
+      <c r="G643" t="inlineStr"/>
+      <c r="H643" t="inlineStr"/>
+      <c r="I643" t="inlineStr">
+        <is>
+          <t>burger</t>
+        </is>
+      </c>
+      <c r="J643" t="inlineStr">
+        <is>
+          <t>Overture Maps category: burger_restaurant (confidence 0.73) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K643" t="inlineStr">
+        <is>
+          <t>other (http://www.kamoraburger.md/)</t>
+        </is>
+      </c>
+      <c r="L643" t="inlineStr"/>
+      <c r="M643" t="n">
+        <v>47.049278</v>
+      </c>
+      <c r="N643" t="n">
+        <v>28.864025</v>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" t="inlineStr">
+        <is>
+          <t>overture/ab976554-d429-4c9e-a0f6-b3270b820260</t>
+        </is>
+      </c>
+      <c r="B644" t="inlineStr">
+        <is>
+          <t>il rosso food truck</t>
+        </is>
+      </c>
+      <c r="C644" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D644" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E644" t="inlineStr">
+        <is>
+          <t>full_meal</t>
+        </is>
+      </c>
+      <c r="F644" t="inlineStr">
+        <is>
+          <t>pizzeria</t>
+        </is>
+      </c>
+      <c r="G644" t="inlineStr"/>
+      <c r="H644" t="inlineStr"/>
+      <c r="I644" t="inlineStr">
+        <is>
+          <t>pizza</t>
+        </is>
+      </c>
+      <c r="J644" t="inlineStr">
+        <is>
+          <t>Overture Maps category: pizza_restaurant (confidence 0.86) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K644" t="inlineStr">
+        <is>
+          <t>other (https://ilrosso.md/)</t>
+        </is>
+      </c>
+      <c r="L644" t="inlineStr"/>
+      <c r="M644" t="n">
+        <v>47.04880101</v>
+      </c>
+      <c r="N644" t="n">
+        <v>28.92778055</v>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" t="inlineStr">
+        <is>
+          <t>overture/86a7e067-2103-4898-9267-ec6500ccc4ae</t>
+        </is>
+      </c>
+      <c r="B645" t="inlineStr">
+        <is>
+          <t>Cerreto</t>
+        </is>
+      </c>
+      <c r="C645" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D645" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E645" t="inlineStr">
+        <is>
+          <t>full_meal</t>
+        </is>
+      </c>
+      <c r="F645" t="inlineStr">
+        <is>
+          <t>pizzeria</t>
+        </is>
+      </c>
+      <c r="G645" t="inlineStr"/>
+      <c r="H645" t="inlineStr"/>
+      <c r="I645" t="inlineStr">
+        <is>
+          <t>pizza</t>
+        </is>
+      </c>
+      <c r="J645" t="inlineStr">
+        <is>
+          <t>Overture Maps category: pizza_restaurant (confidence 0.54) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K645" t="inlineStr">
+        <is>
+          <t>other (http://ceretto.md)</t>
+        </is>
+      </c>
+      <c r="L645" t="inlineStr"/>
+      <c r="M645" t="n">
+        <v>47.038281109523</v>
+      </c>
+      <c r="N645" t="n">
+        <v>28.890223503113</v>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" t="inlineStr">
+        <is>
+          <t>overture/0679f8ea-53fa-40e3-b470-c93b9a988718</t>
+        </is>
+      </c>
+      <c r="B646" t="inlineStr">
+        <is>
+          <t>Toyland</t>
+        </is>
+      </c>
+      <c r="C646" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D646" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E646" t="inlineStr">
+        <is>
+          <t>full_meal</t>
+        </is>
+      </c>
+      <c r="F646" t="inlineStr">
+        <is>
+          <t>pizzeria</t>
+        </is>
+      </c>
+      <c r="G646" t="inlineStr"/>
+      <c r="H646" t="inlineStr"/>
+      <c r="I646" t="inlineStr">
+        <is>
+          <t>pizza</t>
+        </is>
+      </c>
+      <c r="J646" t="inlineStr">
+        <is>
+          <t>Overture Maps category: pizza_restaurant (confidence 0.93) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K646" t="inlineStr">
+        <is>
+          <t>other (https://www.toyland.md)</t>
+        </is>
+      </c>
+      <c r="L646" t="inlineStr"/>
+      <c r="M646" t="n">
+        <v>47.037521</v>
+      </c>
+      <c r="N646" t="n">
+        <v>28.890757</v>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" t="inlineStr">
+        <is>
+          <t>overture/6348c731-0e19-40e4-8fbd-dbe98dedc281</t>
+        </is>
+      </c>
+      <c r="B647" t="inlineStr">
+        <is>
+          <t>Quattro Stagioni</t>
+        </is>
+      </c>
+      <c r="C647" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D647" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E647" t="inlineStr">
+        <is>
+          <t>full_meal</t>
+        </is>
+      </c>
+      <c r="F647" t="inlineStr">
+        <is>
+          <t>pizzeria</t>
+        </is>
+      </c>
+      <c r="G647" t="inlineStr"/>
+      <c r="H647" t="inlineStr"/>
+      <c r="I647" t="inlineStr">
+        <is>
+          <t>pizza</t>
+        </is>
+      </c>
+      <c r="J647" t="inlineStr">
+        <is>
+          <t>Overture Maps category: pizza_restaurant (confidence 0.61) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K647" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="L647" t="inlineStr"/>
+      <c r="M647" t="n">
+        <v>47.03282002</v>
+      </c>
+      <c r="N647" t="n">
+        <v>28.87880159</v>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" t="inlineStr">
+        <is>
+          <t>overture/879bf2e9-ad09-4282-965d-15000033817f</t>
+        </is>
+      </c>
+      <c r="B648" t="inlineStr">
+        <is>
+          <t>Burger Craft</t>
+        </is>
+      </c>
+      <c r="C648" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D648" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E648" t="inlineStr">
+        <is>
+          <t>limited_meal</t>
+        </is>
+      </c>
+      <c r="F648" t="inlineStr">
+        <is>
+          <t>burger_shop</t>
+        </is>
+      </c>
+      <c r="G648" t="inlineStr"/>
+      <c r="H648" t="inlineStr"/>
+      <c r="I648" t="inlineStr">
+        <is>
+          <t>burger</t>
+        </is>
+      </c>
+      <c r="J648" t="inlineStr">
+        <is>
+          <t>Overture Maps category: burger_restaurant (confidence 0.97) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K648" t="inlineStr">
+        <is>
+          <t>other (https://www.burgercraft.md/)</t>
+        </is>
+      </c>
+      <c r="L648" t="inlineStr"/>
+      <c r="M648" t="n">
+        <v>47.030398</v>
+      </c>
+      <c r="N648" t="n">
+        <v>28.839068</v>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" t="inlineStr">
+        <is>
+          <t>overture/5a683176-c6a4-4ae5-82ec-5e5fedb7cb23</t>
+        </is>
+      </c>
+      <c r="B649" t="inlineStr">
+        <is>
+          <t>Masquerade turkish mangal</t>
+        </is>
+      </c>
+      <c r="C649" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D649" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E649" t="inlineStr">
+        <is>
+          <t>full_meal</t>
+        </is>
+      </c>
+      <c r="F649" t="inlineStr">
+        <is>
+          <t>pizzeria</t>
+        </is>
+      </c>
+      <c r="G649" t="inlineStr"/>
+      <c r="H649" t="inlineStr"/>
+      <c r="I649" t="inlineStr">
+        <is>
+          <t>pizza</t>
+        </is>
+      </c>
+      <c r="J649" t="inlineStr">
+        <is>
+          <t>Overture Maps category: pizza_restaurant (confidence 0.89) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K649" t="inlineStr">
+        <is>
+          <t>other (http://www.masquerade.md/)</t>
+        </is>
+      </c>
+      <c r="L649" t="inlineStr"/>
+      <c r="M649" t="n">
+        <v>47.031129685613</v>
+      </c>
+      <c r="N649" t="n">
+        <v>28.822009563446</v>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" t="inlineStr">
+        <is>
+          <t>overture/3f411d6a-e108-4f94-a28e-f5e8c8927b20</t>
+        </is>
+      </c>
+      <c r="B650" t="inlineStr">
+        <is>
+          <t>SAKURA sushi-bar</t>
+        </is>
+      </c>
+      <c r="C650" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D650" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E650" t="inlineStr">
+        <is>
+          <t>full_meal</t>
+        </is>
+      </c>
+      <c r="F650" t="inlineStr">
+        <is>
+          <t>sushi_restaurant</t>
+        </is>
+      </c>
+      <c r="G650" t="inlineStr"/>
+      <c r="H650" t="inlineStr"/>
+      <c r="I650" t="inlineStr">
+        <is>
+          <t>sushi</t>
+        </is>
+      </c>
+      <c r="J650" t="inlineStr">
+        <is>
+          <t>Overture Maps category: sushi_restaurant (confidence 0.54) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K650" t="inlineStr">
+        <is>
+          <t>other (http://sakura.md/ro/)</t>
+        </is>
+      </c>
+      <c r="L650" t="inlineStr"/>
+      <c r="M650" t="n">
+        <v>47.0261</v>
+      </c>
+      <c r="N650" t="n">
+        <v>28.85313</v>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" t="inlineStr">
+        <is>
+          <t>overture/a5e009a1-e1fb-43f9-918b-022c4a3cd7e8</t>
+        </is>
+      </c>
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>Pizza Régal</t>
+        </is>
+      </c>
+      <c r="C651" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D651" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E651" t="inlineStr">
+        <is>
+          <t>full_meal</t>
+        </is>
+      </c>
+      <c r="F651" t="inlineStr">
+        <is>
+          <t>pizzeria</t>
+        </is>
+      </c>
+      <c r="G651" t="inlineStr"/>
+      <c r="H651" t="inlineStr"/>
+      <c r="I651" t="inlineStr">
+        <is>
+          <t>pizza</t>
+        </is>
+      </c>
+      <c r="J651" t="inlineStr">
+        <is>
+          <t>Overture Maps category: pizza_restaurant (confidence 0.71) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K651" t="inlineStr">
+        <is>
+          <t>other (http://pizzaregal.sitew.com/)</t>
+        </is>
+      </c>
+      <c r="L651" t="inlineStr"/>
+      <c r="M651" t="n">
+        <v>47.02583581047634</v>
+      </c>
+      <c r="N651" t="n">
+        <v>28.83173570881285</v>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" t="inlineStr">
+        <is>
+          <t>overture/cb07d6c5-c746-4e24-961d-56b1040bf4da</t>
+        </is>
+      </c>
+      <c r="B652" t="inlineStr">
+        <is>
+          <t>Пицца Мания</t>
+        </is>
+      </c>
+      <c r="C652" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D652" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E652" t="inlineStr">
+        <is>
+          <t>full_meal</t>
+        </is>
+      </c>
+      <c r="F652" t="inlineStr">
+        <is>
+          <t>pizzeria</t>
+        </is>
+      </c>
+      <c r="G652" t="inlineStr"/>
+      <c r="H652" t="inlineStr"/>
+      <c r="I652" t="inlineStr">
+        <is>
+          <t>pizza</t>
+        </is>
+      </c>
+      <c r="J652" t="inlineStr">
+        <is>
+          <t>Overture Maps category: pizza_restaurant (confidence 0.94) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K652" t="inlineStr">
+        <is>
+          <t>other (http://www.pizzamania.md/ro/locatii/pizza-mania-700-0100-b%C4%83nulescu-bodoni)</t>
+        </is>
+      </c>
+      <c r="L652" t="inlineStr"/>
+      <c r="M652" t="n">
+        <v>47.02674182969725</v>
+      </c>
+      <c r="N652" t="n">
+        <v>28.83279193753859</v>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" t="inlineStr">
+        <is>
+          <t>overture/d7051815-c15e-433a-bae5-55bf658b5d69</t>
+        </is>
+      </c>
+      <c r="B653" t="inlineStr">
+        <is>
+          <t>Cinema Patria</t>
+        </is>
+      </c>
+      <c r="C653" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D653" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E653" t="inlineStr">
+        <is>
+          <t>full_meal</t>
+        </is>
+      </c>
+      <c r="F653" t="inlineStr">
+        <is>
+          <t>pizzeria; sushi_restaurant</t>
+        </is>
+      </c>
+      <c r="G653" t="inlineStr"/>
+      <c r="H653" t="inlineStr"/>
+      <c r="I653" t="inlineStr">
+        <is>
+          <t>pizza; sushi</t>
+        </is>
+      </c>
+      <c r="J653" t="inlineStr">
+        <is>
+          <t>Overture Maps category: pizza_restaurant, sushi_restaurant (confidence 0.98) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K653" t="inlineStr">
+        <is>
+          <t>other (https://patria.md/)</t>
+        </is>
+      </c>
+      <c r="L653" t="inlineStr"/>
+      <c r="M653" t="n">
+        <v>47.02701279243934</v>
+      </c>
+      <c r="N653" t="n">
+        <v>28.82841572949087</v>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" t="inlineStr">
+        <is>
+          <t>overture/c7cc4ef8-6738-43b6-8cb5-b62ae0a6e195</t>
+        </is>
+      </c>
+      <c r="B654" t="inlineStr">
+        <is>
+          <t>Moldovainvest</t>
+        </is>
+      </c>
+      <c r="C654" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D654" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E654" t="inlineStr">
+        <is>
+          <t>full_meal</t>
+        </is>
+      </c>
+      <c r="F654" t="inlineStr">
+        <is>
+          <t>pizzeria</t>
+        </is>
+      </c>
+      <c r="G654" t="inlineStr"/>
+      <c r="H654" t="inlineStr"/>
+      <c r="I654" t="inlineStr">
+        <is>
+          <t>pizza</t>
+        </is>
+      </c>
+      <c r="J654" t="inlineStr">
+        <is>
+          <t>Overture Maps category: pizza_restaurant (confidence 0.85) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K654" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="L654" t="inlineStr"/>
+      <c r="M654" t="n">
+        <v>47.0335</v>
+      </c>
+      <c r="N654" t="n">
+        <v>28.83403</v>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" t="inlineStr">
+        <is>
+          <t>overture/bd0e2710-61eb-4312-8a8f-c61701380f83</t>
+        </is>
+      </c>
+      <c r="B655" t="inlineStr">
+        <is>
+          <t>Drugoe Mesto Fast Food</t>
+        </is>
+      </c>
+      <c r="C655" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D655" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E655" t="inlineStr">
+        <is>
+          <t>limited_meal</t>
+        </is>
+      </c>
+      <c r="F655" t="inlineStr">
+        <is>
+          <t>burger_shop</t>
+        </is>
+      </c>
+      <c r="G655" t="inlineStr"/>
+      <c r="H655" t="inlineStr"/>
+      <c r="I655" t="inlineStr">
+        <is>
+          <t>burger</t>
+        </is>
+      </c>
+      <c r="J655" t="inlineStr">
+        <is>
+          <t>Overture Maps category: burger_restaurant (confidence 0.53) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K655" t="inlineStr">
+        <is>
+          <t>other (https://www.straus.md/ru/?query=Drugoe+Mesto)</t>
+        </is>
+      </c>
+      <c r="L655" t="inlineStr"/>
+      <c r="M655" t="n">
+        <v>47.0352595</v>
+      </c>
+      <c r="N655" t="n">
+        <v>28.8482935</v>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" t="inlineStr">
+        <is>
+          <t>overture/f9ab17ac-4d7f-425a-a4a5-bab216f11472</t>
+        </is>
+      </c>
+      <c r="B656" t="inlineStr">
+        <is>
+          <t>Moon_Bar_Lounges</t>
+        </is>
+      </c>
+      <c r="C656" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D656" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E656" t="inlineStr">
+        <is>
+          <t>full_meal</t>
+        </is>
+      </c>
+      <c r="F656" t="inlineStr">
+        <is>
+          <t>sushi_restaurant</t>
+        </is>
+      </c>
+      <c r="G656" t="inlineStr"/>
+      <c r="H656" t="inlineStr"/>
+      <c r="I656" t="inlineStr">
+        <is>
+          <t>sushi</t>
+        </is>
+      </c>
+      <c r="J656" t="inlineStr">
+        <is>
+          <t>Overture Maps category: sushi_restaurant (confidence 0.83) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K656" t="inlineStr">
+        <is>
+          <t>other (https://www.straus.md/ru/restaurant/moon-bar/)</t>
+        </is>
+      </c>
+      <c r="L656" t="inlineStr"/>
+      <c r="M656" t="n">
+        <v>47.03579</v>
+      </c>
+      <c r="N656" t="n">
+        <v>28.8354</v>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" t="inlineStr">
+        <is>
+          <t>overture/b7fec2e6-d056-4aa4-b27d-cc227131e44e</t>
+        </is>
+      </c>
+      <c r="B657" t="inlineStr">
+        <is>
+          <t>Pizza Delice</t>
+        </is>
+      </c>
+      <c r="C657" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D657" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E657" t="inlineStr">
+        <is>
+          <t>full_meal</t>
+        </is>
+      </c>
+      <c r="F657" t="inlineStr">
+        <is>
+          <t>pizzeria</t>
+        </is>
+      </c>
+      <c r="G657" t="inlineStr"/>
+      <c r="H657" t="inlineStr"/>
+      <c r="I657" t="inlineStr">
+        <is>
+          <t>pizza</t>
+        </is>
+      </c>
+      <c r="J657" t="inlineStr">
+        <is>
+          <t>Overture Maps category: pizza_restaurant (confidence 0.94) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K657" t="inlineStr">
+        <is>
+          <t>other (http://delice.md/)</t>
+        </is>
+      </c>
+      <c r="L657" t="inlineStr"/>
+      <c r="M657" t="n">
+        <v>47.03912992</v>
+      </c>
+      <c r="N657" t="n">
+        <v>28.83218774</v>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" t="inlineStr">
+        <is>
+          <t>overture/1441c315-add9-4a73-aee7-b01790e7b501</t>
+        </is>
+      </c>
+      <c r="B658" t="inlineStr">
+        <is>
+          <t>Sushiookami</t>
+        </is>
+      </c>
+      <c r="C658" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D658" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E658" t="inlineStr">
+        <is>
+          <t>full_meal</t>
+        </is>
+      </c>
+      <c r="F658" t="inlineStr">
+        <is>
+          <t>sushi_restaurant</t>
+        </is>
+      </c>
+      <c r="G658" t="inlineStr"/>
+      <c r="H658" t="inlineStr"/>
+      <c r="I658" t="inlineStr">
+        <is>
+          <t>sushi</t>
+        </is>
+      </c>
+      <c r="J658" t="inlineStr">
+        <is>
+          <t>Overture Maps category: sushi_restaurant (confidence 0.53) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K658" t="inlineStr">
+        <is>
+          <t>other (http://ookami.md/)</t>
+        </is>
+      </c>
+      <c r="L658" t="inlineStr"/>
+      <c r="M658" t="n">
+        <v>47.03889895342</v>
+      </c>
+      <c r="N658" t="n">
+        <v>28.830340504646</v>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" t="inlineStr">
+        <is>
+          <t>overture/c1b7ee86-3918-4d8d-996a-b075942534e9</t>
+        </is>
+      </c>
+      <c r="B659" t="inlineStr">
+        <is>
+          <t>Don Cezar Pizza &amp; Grill</t>
+        </is>
+      </c>
+      <c r="C659" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D659" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E659" t="inlineStr">
+        <is>
+          <t>full_meal</t>
+        </is>
+      </c>
+      <c r="F659" t="inlineStr">
+        <is>
+          <t>pizzeria</t>
+        </is>
+      </c>
+      <c r="G659" t="inlineStr"/>
+      <c r="H659" t="inlineStr"/>
+      <c r="I659" t="inlineStr">
+        <is>
+          <t>pizza</t>
+        </is>
+      </c>
+      <c r="J659" t="inlineStr">
+        <is>
+          <t>Overture Maps category: pizza_restaurant (confidence 0.64) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K659" t="inlineStr">
+        <is>
+          <t>other (https://doncezar.md)</t>
+        </is>
+      </c>
+      <c r="L659" t="inlineStr"/>
+      <c r="M659" t="n">
+        <v>47.038901</v>
+      </c>
+      <c r="N659" t="n">
+        <v>28.805334</v>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" t="inlineStr">
+        <is>
+          <t>overture/ae39921e-d6e3-4442-8143-88805a36c921</t>
+        </is>
+      </c>
+      <c r="B660" t="inlineStr">
+        <is>
+          <t>Pepperoni Pizza</t>
+        </is>
+      </c>
+      <c r="C660" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D660" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E660" t="inlineStr">
+        <is>
+          <t>full_meal</t>
+        </is>
+      </c>
+      <c r="F660" t="inlineStr">
+        <is>
+          <t>pizzeria</t>
+        </is>
+      </c>
+      <c r="G660" t="inlineStr"/>
+      <c r="H660" t="inlineStr"/>
+      <c r="I660" t="inlineStr">
+        <is>
+          <t>pizza</t>
+        </is>
+      </c>
+      <c r="J660" t="inlineStr">
+        <is>
+          <t>Overture Maps category: pizza_restaurant (confidence 0.89) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K660" t="inlineStr">
+        <is>
+          <t>other (https://glovoapp.com/md/ro/chisinau/pepperoni-pizza/)</t>
+        </is>
+      </c>
+      <c r="L660" t="inlineStr"/>
+      <c r="M660" t="n">
+        <v>47.03877843</v>
+      </c>
+      <c r="N660" t="n">
+        <v>28.80445348</v>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" t="inlineStr">
+        <is>
+          <t>overture/f630796c-69cd-4a94-81b6-5a734b172644</t>
+        </is>
+      </c>
+      <c r="B661" t="inlineStr">
+        <is>
+          <t>Pegas Burger Cafe</t>
+        </is>
+      </c>
+      <c r="C661" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D661" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E661" t="inlineStr">
+        <is>
+          <t>limited_meal</t>
+        </is>
+      </c>
+      <c r="F661" t="inlineStr">
+        <is>
+          <t>burger_shop</t>
+        </is>
+      </c>
+      <c r="G661" t="inlineStr"/>
+      <c r="H661" t="inlineStr"/>
+      <c r="I661" t="inlineStr">
+        <is>
+          <t>burger</t>
+        </is>
+      </c>
+      <c r="J661" t="inlineStr">
+        <is>
+          <t>Overture Maps category: burger_restaurant (confidence 0.95) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K661" t="inlineStr">
+        <is>
+          <t>other (https://og-burger.md/)</t>
+        </is>
+      </c>
+      <c r="L661" t="inlineStr"/>
+      <c r="M661" t="n">
+        <v>47.03841431</v>
+      </c>
+      <c r="N661" t="n">
+        <v>28.8124106</v>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" t="inlineStr">
+        <is>
+          <t>overture/d60fd42a-cd85-4a35-a9af-5c8f0389e79b</t>
+        </is>
+      </c>
+      <c r="B662" t="inlineStr">
+        <is>
+          <t>Nakiri Sushi</t>
+        </is>
+      </c>
+      <c r="C662" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D662" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E662" t="inlineStr">
+        <is>
+          <t>full_meal</t>
+        </is>
+      </c>
+      <c r="F662" t="inlineStr">
+        <is>
+          <t>sushi_restaurant</t>
+        </is>
+      </c>
+      <c r="G662" t="inlineStr"/>
+      <c r="H662" t="inlineStr"/>
+      <c r="I662" t="inlineStr">
+        <is>
+          <t>sushi</t>
+        </is>
+      </c>
+      <c r="J662" t="inlineStr">
+        <is>
+          <t>Overture Maps category: sushi_restaurant (confidence 0.83) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K662" t="inlineStr">
+        <is>
+          <t>other (https://senseisushi.md/ru)</t>
+        </is>
+      </c>
+      <c r="L662" t="inlineStr"/>
+      <c r="M662" t="n">
+        <v>47.03803533</v>
+      </c>
+      <c r="N662" t="n">
+        <v>28.77511254</v>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" t="inlineStr">
+        <is>
+          <t>overture/8463d511-5aa7-4d53-a0b8-8dd23e215204</t>
+        </is>
+      </c>
+      <c r="B663" t="inlineStr">
+        <is>
+          <t>Pizzeria pe vatră</t>
+        </is>
+      </c>
+      <c r="C663" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D663" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E663" t="inlineStr">
+        <is>
+          <t>full_meal</t>
+        </is>
+      </c>
+      <c r="F663" t="inlineStr">
+        <is>
+          <t>pizzeria</t>
+        </is>
+      </c>
+      <c r="G663" t="inlineStr"/>
+      <c r="H663" t="inlineStr"/>
+      <c r="I663" t="inlineStr">
+        <is>
+          <t>pizza</t>
+        </is>
+      </c>
+      <c r="J663" t="inlineStr">
+        <is>
+          <t>Overture Maps category: pizza_restaurant (confidence 0.93) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K663" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="L663" t="inlineStr"/>
+      <c r="M663" t="n">
+        <v>47.03984896</v>
+      </c>
+      <c r="N663" t="n">
+        <v>28.74101193</v>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" t="inlineStr">
+        <is>
+          <t>overture/871389e7-6cdd-43e1-8bea-71efc765e5dc</t>
+        </is>
+      </c>
+      <c r="B664" t="inlineStr">
+        <is>
+          <t>Super Kebab</t>
+        </is>
+      </c>
+      <c r="C664" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D664" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E664" t="inlineStr">
+        <is>
+          <t>limited_meal</t>
+        </is>
+      </c>
+      <c r="F664" t="inlineStr">
+        <is>
+          <t>burger_shop; kebab_shop</t>
+        </is>
+      </c>
+      <c r="G664" t="inlineStr"/>
+      <c r="H664" t="inlineStr"/>
+      <c r="I664" t="inlineStr">
+        <is>
+          <t>burger; kebab</t>
+        </is>
+      </c>
+      <c r="J664" t="inlineStr">
+        <is>
+          <t>Overture Maps category: burger_restaurant, doner_kebab (confidence 0.81) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K664" t="inlineStr">
+        <is>
+          <t>other (http://www.damaskos.simplesite.com/)</t>
+        </is>
+      </c>
+      <c r="L664" t="inlineStr"/>
+      <c r="M664" t="n">
+        <v>47.02754014</v>
+      </c>
+      <c r="N664" t="n">
+        <v>28.7717174</v>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" t="inlineStr">
+        <is>
+          <t>overture/e0deaa95-19b7-436f-b3d2-977803dee9ec</t>
+        </is>
+      </c>
+      <c r="B665" t="inlineStr">
+        <is>
+          <t>ODIS Pizza</t>
+        </is>
+      </c>
+      <c r="C665" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D665" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E665" t="inlineStr">
+        <is>
+          <t>full_meal</t>
+        </is>
+      </c>
+      <c r="F665" t="inlineStr">
+        <is>
+          <t>pizzeria</t>
+        </is>
+      </c>
+      <c r="G665" t="inlineStr"/>
+      <c r="H665" t="inlineStr"/>
+      <c r="I665" t="inlineStr">
+        <is>
+          <t>pizza</t>
+        </is>
+      </c>
+      <c r="J665" t="inlineStr">
+        <is>
+          <t>Overture Maps category: pizza_restaurant (confidence 0.93) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K665" t="inlineStr">
+        <is>
+          <t>other (https://glovoapp.com/md/en/chisinau/odis-pizza-md/)</t>
+        </is>
+      </c>
+      <c r="L665" t="inlineStr"/>
+      <c r="M665" t="n">
+        <v>47.0150306</v>
+      </c>
+      <c r="N665" t="n">
+        <v>28.74781218</v>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" t="inlineStr">
+        <is>
+          <t>overture/b4663e43-b1d4-4fb0-844a-5bd00b58d743</t>
+        </is>
+      </c>
+      <c r="B666" t="inlineStr">
+        <is>
+          <t>Andy's Pizza</t>
+        </is>
+      </c>
+      <c r="C666" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D666" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E666" t="inlineStr">
+        <is>
+          <t>full_meal</t>
+        </is>
+      </c>
+      <c r="F666" t="inlineStr">
+        <is>
+          <t>pizzeria</t>
+        </is>
+      </c>
+      <c r="G666" t="inlineStr"/>
+      <c r="H666" t="inlineStr"/>
+      <c r="I666" t="inlineStr">
+        <is>
+          <t>pizza</t>
+        </is>
+      </c>
+      <c r="J666" t="inlineStr">
+        <is>
+          <t>Overture Maps category: pizza_restaurant (confidence 0.77) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K666" t="inlineStr">
+        <is>
+          <t>other (https://www.andys.md)</t>
+        </is>
+      </c>
+      <c r="L666" t="inlineStr"/>
+      <c r="M666" t="n">
+        <v>47.00709080848264</v>
+      </c>
+      <c r="N666" t="n">
+        <v>28.76411408185959</v>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" t="inlineStr">
+        <is>
+          <t>overture/dcf2a9db-fe61-4083-8fe5-8af206f51116</t>
+        </is>
+      </c>
+      <c r="B667" t="inlineStr">
+        <is>
+          <t>ВышеГор</t>
+        </is>
+      </c>
+      <c r="C667" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D667" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E667" t="inlineStr">
+        <is>
+          <t>full_meal</t>
+        </is>
+      </c>
+      <c r="F667" t="inlineStr">
+        <is>
+          <t>sushi_restaurant</t>
+        </is>
+      </c>
+      <c r="G667" t="inlineStr"/>
+      <c r="H667" t="inlineStr"/>
+      <c r="I667" t="inlineStr">
+        <is>
+          <t>sushi</t>
+        </is>
+      </c>
+      <c r="J667" t="inlineStr">
+        <is>
+          <t>Overture Maps category: sushi_restaurant (confidence 0.88) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K667" t="inlineStr">
+        <is>
+          <t>other (http://www.instagram.com/vishefudzi/?hl=ru)</t>
+        </is>
+      </c>
+      <c r="L667" t="inlineStr"/>
+      <c r="M667" t="n">
+        <v>47.00619433</v>
+      </c>
+      <c r="N667" t="n">
+        <v>28.82636712</v>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" t="inlineStr">
+        <is>
+          <t>overture/af4bbec3-d454-46dc-9d81-b85304f6d81a</t>
+        </is>
+      </c>
+      <c r="B668" t="inlineStr">
+        <is>
+          <t>Corso Pizza</t>
+        </is>
+      </c>
+      <c r="C668" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D668" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E668" t="inlineStr">
+        <is>
+          <t>full_meal</t>
+        </is>
+      </c>
+      <c r="F668" t="inlineStr">
+        <is>
+          <t>pizzeria</t>
+        </is>
+      </c>
+      <c r="G668" t="inlineStr"/>
+      <c r="H668" t="inlineStr"/>
+      <c r="I668" t="inlineStr">
+        <is>
+          <t>pizza</t>
+        </is>
+      </c>
+      <c r="J668" t="inlineStr">
+        <is>
+          <t>Overture Maps category: pizza_restaurant (confidence 0.95) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K668" t="inlineStr">
+        <is>
+          <t>other (http://www.corso.md/)</t>
+        </is>
+      </c>
+      <c r="L668" t="inlineStr"/>
+      <c r="M668" t="n">
+        <v>47.00800062</v>
+      </c>
+      <c r="N668" t="n">
+        <v>28.83220435</v>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" t="inlineStr">
+        <is>
+          <t>overture/f8a58cce-7d3f-459b-9a7f-c93544a4383e</t>
+        </is>
+      </c>
+      <c r="B669" t="inlineStr">
+        <is>
+          <t>Samurai Sushi and Rolls</t>
+        </is>
+      </c>
+      <c r="C669" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D669" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E669" t="inlineStr">
+        <is>
+          <t>full_meal</t>
+        </is>
+      </c>
+      <c r="F669" t="inlineStr">
+        <is>
+          <t>sushi_restaurant</t>
+        </is>
+      </c>
+      <c r="G669" t="inlineStr"/>
+      <c r="H669" t="inlineStr"/>
+      <c r="I669" t="inlineStr">
+        <is>
+          <t>sushi</t>
+        </is>
+      </c>
+      <c r="J669" t="inlineStr">
+        <is>
+          <t>Overture Maps category: sushi_restaurant (confidence 0.65) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K669" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="L669" t="inlineStr"/>
+      <c r="M669" t="n">
+        <v>47.01357165</v>
+      </c>
+      <c r="N669" t="n">
+        <v>28.85633523</v>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" t="inlineStr">
+        <is>
+          <t>overture/43857500-10ee-43e8-9375-536fff263023</t>
+        </is>
+      </c>
+      <c r="B670" t="inlineStr">
+        <is>
+          <t>RiceNRoll</t>
+        </is>
+      </c>
+      <c r="C670" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D670" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E670" t="inlineStr">
+        <is>
+          <t>full_meal</t>
+        </is>
+      </c>
+      <c r="F670" t="inlineStr">
+        <is>
+          <t>sushi_restaurant</t>
+        </is>
+      </c>
+      <c r="G670" t="inlineStr"/>
+      <c r="H670" t="inlineStr"/>
+      <c r="I670" t="inlineStr">
+        <is>
+          <t>sushi</t>
+        </is>
+      </c>
+      <c r="J670" t="inlineStr">
+        <is>
+          <t>Overture Maps category: sushi_restaurant (confidence 0.89) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K670" t="inlineStr">
+        <is>
+          <t>other (https://glovoapp.com/md/ro/chisinau/rice-n-roll/)</t>
+        </is>
+      </c>
+      <c r="L670" t="inlineStr"/>
+      <c r="M670" t="n">
+        <v>47.01997142</v>
+      </c>
+      <c r="N670" t="n">
+        <v>28.79520917</v>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" t="inlineStr">
+        <is>
+          <t>overture/6fda8a48-0cab-4112-9ed0-95f960185c66</t>
+        </is>
+      </c>
+      <c r="B671" t="inlineStr">
+        <is>
+          <t>Gusto Italiano Ristorante</t>
+        </is>
+      </c>
+      <c r="C671" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D671" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E671" t="inlineStr">
+        <is>
+          <t>full_meal</t>
+        </is>
+      </c>
+      <c r="F671" t="inlineStr">
+        <is>
+          <t>pizzeria</t>
+        </is>
+      </c>
+      <c r="G671" t="inlineStr"/>
+      <c r="H671" t="inlineStr"/>
+      <c r="I671" t="inlineStr">
+        <is>
+          <t>pizza</t>
+        </is>
+      </c>
+      <c r="J671" t="inlineStr">
+        <is>
+          <t>Overture Maps category: pizza_restaurant (confidence 0.99) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K671" t="inlineStr">
+        <is>
+          <t>other (http://www.gustoristo.md/)</t>
+        </is>
+      </c>
+      <c r="L671" t="inlineStr"/>
+      <c r="M671" t="n">
+        <v>47.01987</v>
+      </c>
+      <c r="N671" t="n">
+        <v>28.82226</v>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" t="inlineStr">
+        <is>
+          <t>overture/b721a0d3-aa7f-458e-ba3f-3036d416d60e</t>
+        </is>
+      </c>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>Pizza Point</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D672" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E672" t="inlineStr">
+        <is>
+          <t>full_meal</t>
+        </is>
+      </c>
+      <c r="F672" t="inlineStr">
+        <is>
+          <t>pizzeria</t>
+        </is>
+      </c>
+      <c r="G672" t="inlineStr"/>
+      <c r="H672" t="inlineStr"/>
+      <c r="I672" t="inlineStr">
+        <is>
+          <t>pizza</t>
+        </is>
+      </c>
+      <c r="J672" t="inlineStr">
+        <is>
+          <t>Overture Maps category: pizza_restaurant (confidence 0.57) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K672" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="L672" t="inlineStr"/>
+      <c r="M672" t="n">
+        <v>47.02093</v>
+      </c>
+      <c r="N672" t="n">
+        <v>28.84067</v>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" t="inlineStr">
+        <is>
+          <t>overture/17cb7466-0f65-430e-b732-9c40a7d44895</t>
+        </is>
+      </c>
+      <c r="B673" t="inlineStr">
+        <is>
+          <t>Atlantis Kebab</t>
+        </is>
+      </c>
+      <c r="C673" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D673" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E673" t="inlineStr">
+        <is>
+          <t>limited_meal</t>
+        </is>
+      </c>
+      <c r="F673" t="inlineStr">
+        <is>
+          <t>kebab_shop</t>
+        </is>
+      </c>
+      <c r="G673" t="inlineStr"/>
+      <c r="H673" t="inlineStr"/>
+      <c r="I673" t="inlineStr">
+        <is>
+          <t>kebab</t>
+        </is>
+      </c>
+      <c r="J673" t="inlineStr">
+        <is>
+          <t>Overture Maps category: doner_kebab (confidence 0.77) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K673" t="inlineStr">
+        <is>
+          <t>other (https://atlantis-kebab.business.site)</t>
+        </is>
+      </c>
+      <c r="L673" t="inlineStr"/>
+      <c r="M673" t="n">
+        <v>47.01959423586907</v>
+      </c>
+      <c r="N673" t="n">
+        <v>28.8448378443718</v>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" t="inlineStr">
+        <is>
+          <t>overture/bcdc76e7-d3f9-4f3b-a6b4-a9d8d1cba177</t>
+        </is>
+      </c>
+      <c r="B674" t="inlineStr">
+        <is>
+          <t>Andys</t>
+        </is>
+      </c>
+      <c r="C674" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D674" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E674" t="inlineStr">
+        <is>
+          <t>full_meal</t>
+        </is>
+      </c>
+      <c r="F674" t="inlineStr">
+        <is>
+          <t>pizzeria</t>
+        </is>
+      </c>
+      <c r="G674" t="inlineStr"/>
+      <c r="H674" t="inlineStr"/>
+      <c r="I674" t="inlineStr">
+        <is>
+          <t>pizza</t>
+        </is>
+      </c>
+      <c r="J674" t="inlineStr">
+        <is>
+          <t>Overture Maps category: pizza_restaurant (confidence 0.95) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K674" t="inlineStr">
+        <is>
+          <t>other (http://andys-pizza.com)</t>
+        </is>
+      </c>
+      <c r="L674" t="inlineStr"/>
+      <c r="M674" t="n">
+        <v>47.01695503</v>
+      </c>
+      <c r="N674" t="n">
+        <v>28.84709475</v>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" t="inlineStr">
+        <is>
+          <t>overture/3fc7828d-1f12-47b4-8d8d-8fdd03af584f</t>
+        </is>
+      </c>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>Ikigai Sushi</t>
+        </is>
+      </c>
+      <c r="C675" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D675" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E675" t="inlineStr">
+        <is>
+          <t>full_meal</t>
+        </is>
+      </c>
+      <c r="F675" t="inlineStr">
+        <is>
+          <t>sushi_restaurant</t>
+        </is>
+      </c>
+      <c r="G675" t="inlineStr"/>
+      <c r="H675" t="inlineStr"/>
+      <c r="I675" t="inlineStr">
+        <is>
+          <t>sushi</t>
+        </is>
+      </c>
+      <c r="J675" t="inlineStr">
+        <is>
+          <t>Overture Maps category: sushi_restaurant (confidence 0.54) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K675" t="inlineStr">
+        <is>
+          <t>other (https://www.ikigaisushi.md/)</t>
+        </is>
+      </c>
+      <c r="L675" t="inlineStr"/>
+      <c r="M675" t="n">
+        <v>47.01486392</v>
+      </c>
+      <c r="N675" t="n">
+        <v>28.8451581</v>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" t="inlineStr">
+        <is>
+          <t>overture/85048742-53fe-42af-afe4-11e5581882b1</t>
+        </is>
+      </c>
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>Pomodoro Pizza Pasta</t>
+        </is>
+      </c>
+      <c r="C676" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D676" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E676" t="inlineStr">
+        <is>
+          <t>full_meal</t>
+        </is>
+      </c>
+      <c r="F676" t="inlineStr">
+        <is>
+          <t>pizzeria</t>
+        </is>
+      </c>
+      <c r="G676" t="inlineStr"/>
+      <c r="H676" t="inlineStr"/>
+      <c r="I676" t="inlineStr">
+        <is>
+          <t>pizza</t>
+        </is>
+      </c>
+      <c r="J676" t="inlineStr">
+        <is>
+          <t>Overture Maps category: pizza_restaurant (confidence 0.82) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K676" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="L676" t="inlineStr"/>
+      <c r="M676" t="n">
+        <v>47.014841630145</v>
+      </c>
+      <c r="N676" t="n">
+        <v>28.855590820313</v>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" t="inlineStr">
+        <is>
+          <t>overture/ed9c1be0-6cf4-406a-b30f-2ef5a92bcbed</t>
+        </is>
+      </c>
+      <c r="B677" t="inlineStr">
+        <is>
+          <t>AkaiSushi Wok</t>
+        </is>
+      </c>
+      <c r="C677" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D677" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E677" t="inlineStr">
+        <is>
+          <t>full_meal</t>
+        </is>
+      </c>
+      <c r="F677" t="inlineStr">
+        <is>
+          <t>sushi_restaurant</t>
+        </is>
+      </c>
+      <c r="G677" t="inlineStr"/>
+      <c r="H677" t="inlineStr"/>
+      <c r="I677" t="inlineStr">
+        <is>
+          <t>sushi</t>
+        </is>
+      </c>
+      <c r="J677" t="inlineStr">
+        <is>
+          <t>Overture Maps category: sushi_restaurant (confidence 0.55) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K677" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="L677" t="inlineStr"/>
+      <c r="M677" t="n">
+        <v>47.014863575188</v>
+      </c>
+      <c r="N677" t="n">
+        <v>28.855719566345</v>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" t="inlineStr">
+        <is>
+          <t>overture/b76b5c31-d6eb-4fa5-80a2-004049b1af5a</t>
+        </is>
+      </c>
+      <c r="B678" t="inlineStr">
+        <is>
+          <t>Pizza Mania</t>
+        </is>
+      </c>
+      <c r="C678" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D678" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E678" t="inlineStr">
+        <is>
+          <t>full_meal</t>
+        </is>
+      </c>
+      <c r="F678" t="inlineStr">
+        <is>
+          <t>pizzeria</t>
+        </is>
+      </c>
+      <c r="G678" t="inlineStr"/>
+      <c r="H678" t="inlineStr"/>
+      <c r="I678" t="inlineStr">
+        <is>
+          <t>pizza</t>
+        </is>
+      </c>
+      <c r="J678" t="inlineStr">
+        <is>
+          <t>Overture Maps category: pizza_restaurant (confidence 0.93) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K678" t="inlineStr">
+        <is>
+          <t>other (https://pizzamania.md/ro/locatii/pizza-mania-baby-hall)</t>
+        </is>
+      </c>
+      <c r="L678" t="inlineStr"/>
+      <c r="M678" t="n">
+        <v>47.01526463</v>
+      </c>
+      <c r="N678" t="n">
+        <v>28.85318562</v>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" t="inlineStr">
+        <is>
+          <t>overture/8bd4bbf1-151c-4f6f-8bdc-624e1a44d735</t>
+        </is>
+      </c>
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>NoriSushi.md</t>
+        </is>
+      </c>
+      <c r="C679" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D679" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E679" t="inlineStr">
+        <is>
+          <t>full_meal</t>
+        </is>
+      </c>
+      <c r="F679" t="inlineStr">
+        <is>
+          <t>sushi_restaurant</t>
+        </is>
+      </c>
+      <c r="G679" t="inlineStr"/>
+      <c r="H679" t="inlineStr"/>
+      <c r="I679" t="inlineStr">
+        <is>
+          <t>sushi</t>
+        </is>
+      </c>
+      <c r="J679" t="inlineStr">
+        <is>
+          <t>Overture Maps category: sushi_restaurant (confidence 0.93) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K679" t="inlineStr">
+        <is>
+          <t>other (http://www.norisushi.md/)</t>
+        </is>
+      </c>
+      <c r="L679" t="inlineStr"/>
+      <c r="M679" t="n">
+        <v>47.02239</v>
+      </c>
+      <c r="N679" t="n">
+        <v>28.87338</v>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" t="inlineStr">
+        <is>
+          <t>overture/1e52033e-100f-4434-99a4-1d3d3cb8dcc5</t>
+        </is>
+      </c>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>Kebab Express</t>
+        </is>
+      </c>
+      <c r="C680" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D680" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E680" t="inlineStr">
+        <is>
+          <t>limited_meal</t>
+        </is>
+      </c>
+      <c r="F680" t="inlineStr">
+        <is>
+          <t>kebab_shop</t>
+        </is>
+      </c>
+      <c r="G680" t="inlineStr"/>
+      <c r="H680" t="inlineStr"/>
+      <c r="I680" t="inlineStr">
+        <is>
+          <t>kebab</t>
+        </is>
+      </c>
+      <c r="J680" t="inlineStr">
+        <is>
+          <t>Overture Maps category: doner_kebab (confidence 0.86) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K680" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="L680" t="inlineStr"/>
+      <c r="M680" t="n">
+        <v>47.00777668</v>
+      </c>
+      <c r="N680" t="n">
+        <v>28.89268854</v>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" t="inlineStr">
+        <is>
+          <t>overture/a1e6c396-c0a9-44d0-9940-9bb740013341</t>
+        </is>
+      </c>
+      <c r="B681" t="inlineStr">
+        <is>
+          <t>Life Cafe</t>
+        </is>
+      </c>
+      <c r="C681" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D681" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E681" t="inlineStr">
+        <is>
+          <t>full_meal</t>
+        </is>
+      </c>
+      <c r="F681" t="inlineStr">
+        <is>
+          <t>pizzeria</t>
+        </is>
+      </c>
+      <c r="G681" t="inlineStr"/>
+      <c r="H681" t="inlineStr"/>
+      <c r="I681" t="inlineStr">
+        <is>
+          <t>pizza</t>
+        </is>
+      </c>
+      <c r="J681" t="inlineStr">
+        <is>
+          <t>Overture Maps category: pizza_restaurant (confidence 0.80) Not present in the original OSM-derived venue list.</t>
+        </is>
+      </c>
+      <c r="K681" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="L681" t="inlineStr"/>
+      <c r="M681" t="n">
+        <v>47.08954521</v>
+      </c>
+      <c r="N681" t="n">
+        <v>28.86446625</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>